<commit_message>
Updating patron_puertos dataset. Minor corrections in identifica_puertos documentation
</commit_message>
<xml_diff>
--- a/inst/extdata/raw-data/coordenadas_caletas.xlsx
+++ b/inst/extdata/raw-data/coordenadas_caletas.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afipdbl\Documents\ruisu\inst\extdata\raw-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afipdbl\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D99772-2732-47ED-9D6E-9C4A7D174AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF6C9BA-F6E0-48EF-9191-E6C79E0E05E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1695" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="puntos_chequeo" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">puntos_chequeo!$A$1:$H$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$73</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -55,7 +55,7 @@
     <t>NORTE</t>
   </si>
   <si>
-    <t>TUMBES</t>
+    <t xml:space="preserve">TUMBES </t>
   </si>
   <si>
     <t>PUERTO 25</t>
@@ -130,7 +130,7 @@
     <t>^(cabo|c)\\.* blanco$</t>
   </si>
   <si>
-    <t>NORTE</t>
+    <t xml:space="preserve">NORTE </t>
   </si>
   <si>
     <t>LOBITOS</t>
@@ -166,6 +166,9 @@
     <t>MATACABALLO</t>
   </si>
   <si>
+    <t>sechura</t>
+  </si>
+  <si>
     <t>matacaballo</t>
   </si>
   <si>
@@ -187,12 +190,15 @@
     <t>parachique</t>
   </si>
   <si>
+    <t>BAYÓVAR</t>
+  </si>
+  <si>
+    <t>^bayovar</t>
+  </si>
+  <si>
     <t>PUERTO RICO</t>
   </si>
   <si>
-    <t>^bayovar</t>
-  </si>
-  <si>
     <t>^(puerto|pto)\\.* rico$</t>
   </si>
   <si>
@@ -232,7 +238,7 @@
     <t>HUANCHACO</t>
   </si>
   <si>
-    <t>LA LIBERTAD</t>
+    <t xml:space="preserve">LA LIBERTAD </t>
   </si>
   <si>
     <t>PACASMAYO</t>
@@ -518,23 +524,27 @@
   </si>
   <si>
     <t>^los palos$</t>
-  </si>
-  <si>
-    <t>sechura</t>
-  </si>
-  <si>
-    <t>BAYÓVAR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -557,14 +567,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -577,9 +590,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -587,44 +600,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -652,31 +665,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -704,26 +700,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -732,207 +711,210 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="1023" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -955,7 +937,7 @@
         <v>-80.270838409999996</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -981,7 +963,7 @@
         <v>-80.389569190000003</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1007,7 +989,7 @@
         <v>-80.587270750000002</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1033,7 +1015,7 @@
         <v>-80.630589139999998</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1059,7 +1041,7 @@
         <v>-80.674713389999994</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1085,7 +1067,7 @@
         <v>-80.773265370000004</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1111,7 +1093,7 @@
         <v>-80.940315589999997</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1137,7 +1119,7 @@
         <v>-81.06745239</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1163,7 +1145,7 @@
         <v>-81.134687450000001</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1189,7 +1171,7 @@
         <v>-81.181357610000006</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1215,7 +1197,7 @@
         <v>-81.230729339999996</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1238,7 +1220,7 @@
         <v>-81.280382509999995</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1264,7 +1246,7 @@
         <v>-81.275349439999999</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1290,7 +1272,7 @@
         <v>-81.113905389999999</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1313,7 +1295,7 @@
         <v>-81.113904520000006</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -1339,7 +1321,7 @@
         <v>-81.171286249999994</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -1365,7 +1347,7 @@
         <v>-81.194560800000005</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1382,7 +1364,7 @@
         <v>46</v>
       </c>
       <c r="F19" t="s">
-        <v>165</v>
+        <v>47</v>
       </c>
       <c r="G19">
         <v>-5.6390510000000003</v>
@@ -1391,7 +1373,7 @@
         <v>-80.850622000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1408,7 +1390,7 @@
         <v>46</v>
       </c>
       <c r="F20" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G20">
         <v>-5.6390510000000003</v>
@@ -1417,7 +1399,7 @@
         <v>-80.850622000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1431,10 +1413,10 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G21">
         <v>-5.6764354099999998</v>
@@ -1443,7 +1425,7 @@
         <v>-80.851046729999993</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -1457,10 +1439,10 @@
         <v>74</v>
       </c>
       <c r="E22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G22">
         <v>-5.7011777600000002</v>
@@ -1469,7 +1451,7 @@
         <v>-80.852360149999996</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1483,10 +1465,10 @@
         <v>13</v>
       </c>
       <c r="E23" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G23">
         <v>-5.7734278699999999</v>
@@ -1495,7 +1477,7 @@
         <v>-80.866036489999999</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -1506,10 +1488,10 @@
         <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>166</v>
+        <v>55</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G24">
         <v>-5.8202444800000004</v>
@@ -1518,7 +1500,7 @@
         <v>-81.036567700000006</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -1532,10 +1514,10 @@
         <v>14</v>
       </c>
       <c r="E25" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G25">
         <v>-5.8202444800000004</v>
@@ -1544,7 +1526,7 @@
         <v>-81.036567700000006</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1555,10 +1537,10 @@
         <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G26">
         <v>-5.8395142399999997</v>
@@ -1567,24 +1549,24 @@
         <v>-80.933867460000002</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D27">
         <v>15</v>
       </c>
       <c r="E27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G27">
         <v>-6.76987337</v>
@@ -1593,24 +1575,24 @@
         <v>-79.972632129999994</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D28">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F28" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G28">
         <v>-6.8393374199999997</v>
@@ -1619,24 +1601,24 @@
         <v>-79.941871109999994</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D29">
         <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F29" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G29">
         <v>-6.8817790499999996</v>
@@ -1645,24 +1627,24 @@
         <v>-79.92329771</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D30">
         <v>71</v>
       </c>
       <c r="E30" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G30">
         <v>-6.9376762799999998</v>
@@ -1671,24 +1653,24 @@
         <v>-79.870230660000004</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D31">
         <v>18</v>
       </c>
       <c r="E31" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F31" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G31">
         <v>-7.3982268199999996</v>
@@ -1697,24 +1679,24 @@
         <v>-79.575033529999999</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D32">
         <v>19</v>
       </c>
       <c r="E32" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F32" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G32">
         <v>-7.6937136099999996</v>
@@ -1723,24 +1705,24 @@
         <v>-79.441239240000002</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D33">
         <v>20</v>
       </c>
       <c r="E33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G33">
         <v>-8.0780522000000001</v>
@@ -1749,24 +1731,24 @@
         <v>-79.120134030000003</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34">
         <v>21</v>
       </c>
       <c r="E34" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G34">
         <v>-8.2239214300000008</v>
@@ -1775,24 +1757,24 @@
         <v>-78.982160480000005</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D35">
         <v>86</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G35">
         <v>-8.3982111499999998</v>
@@ -1801,21 +1783,21 @@
         <v>-78.899751499999994</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G36">
         <v>-8.9913039999999995</v>
@@ -1824,24 +1806,24 @@
         <v>-78.651668000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D37">
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G37">
         <v>-9.07711617</v>
@@ -1850,24 +1832,24 @@
         <v>-78.60114738</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C38" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D38">
         <v>73</v>
       </c>
       <c r="E38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F38" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G38">
         <v>-9.18834996</v>
@@ -1876,21 +1858,21 @@
         <v>-78.564763990000003</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E39" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G39">
         <v>-9.2544988700000008</v>
@@ -1899,24 +1881,24 @@
         <v>-78.500025489999999</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C40" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D40">
         <v>23</v>
       </c>
       <c r="E40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G40">
         <v>-9.3280854699999995</v>
@@ -1925,24 +1907,24 @@
         <v>-78.472633729999998</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C41" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D41">
         <v>55</v>
       </c>
       <c r="E41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F41" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G41">
         <v>-9.4559849699999994</v>
@@ -1951,24 +1933,24 @@
         <v>-78.38601457</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C42" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D42">
         <v>25</v>
       </c>
       <c r="E42" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F42" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G42">
         <v>-9.9485368100000002</v>
@@ -1977,21 +1959,21 @@
         <v>-78.22910238</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E43" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F43" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G43">
         <v>-10.09690239</v>
@@ -2000,24 +1982,24 @@
         <v>-78.17171012</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B44" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D44">
         <v>52</v>
       </c>
       <c r="E44" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F44" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G44">
         <v>-10.79886449</v>
@@ -2026,24 +2008,24 @@
         <v>-77.747532989999996</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C45" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D45">
         <v>53</v>
       </c>
       <c r="E45" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F45" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G45">
         <v>-11.00651332</v>
@@ -2052,24 +2034,24 @@
         <v>-77.655047539999998</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D46">
         <v>26</v>
       </c>
       <c r="E46" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F46" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G46">
         <v>-11.090940249999999</v>
@@ -2078,24 +2060,24 @@
         <v>-77.629084149999997</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D47">
         <v>27</v>
       </c>
       <c r="E47" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F47" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G47">
         <v>-11.12148358</v>
@@ -2104,24 +2086,24 @@
         <v>-77.617495020000007</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C48" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D48">
         <v>28</v>
       </c>
       <c r="E48" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F48" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G48">
         <v>-11.58407182</v>
@@ -2130,24 +2112,24 @@
         <v>-77.273581250000007</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B49" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C49" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D49">
         <v>29</v>
       </c>
       <c r="E49" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F49" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G49">
         <v>-11.77297877</v>
@@ -2156,24 +2138,24 @@
         <v>-77.176677830000003</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B50" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D50">
         <v>30</v>
       </c>
       <c r="E50" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F50" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G50">
         <v>-12.04542687</v>
@@ -2182,24 +2164,24 @@
         <v>-77.141302440000004</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B51" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D51">
         <v>31</v>
       </c>
       <c r="E51" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F51" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G51">
         <v>-12.16430107</v>
@@ -2208,24 +2190,24 @@
         <v>-77.030359840000003</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D52">
         <v>32</v>
       </c>
       <c r="E52" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F52" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G52">
         <v>-12.48003514</v>
@@ -2234,24 +2216,24 @@
         <v>-76.799656150000004</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C53" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D53">
         <v>33</v>
       </c>
       <c r="E53" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F53" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G53">
         <v>-13.02704005</v>
@@ -2260,24 +2242,24 @@
         <v>-76.483065089999997</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B54" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C54" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D54">
         <v>34</v>
       </c>
       <c r="E54" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F54" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G54">
         <v>-13.471300640000001</v>
@@ -2286,24 +2268,24 @@
         <v>-76.192710930000004</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B55" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C55" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D55">
         <v>35</v>
       </c>
       <c r="E55" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F55" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G55">
         <v>-13.733026690000001</v>
@@ -2312,24 +2294,24 @@
         <v>-76.225342560000001</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B56" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C56" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D56">
         <v>81</v>
       </c>
       <c r="E56" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F56" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G56">
         <v>-13.819647209999999</v>
@@ -2338,24 +2320,24 @@
         <v>-76.251748890000002</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B57" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C57" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D57">
         <v>36</v>
       </c>
       <c r="E57" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F57" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G57">
         <v>-13.83204666</v>
@@ -2364,24 +2346,24 @@
         <v>-76.249315699999997</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B58" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C58" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D58">
         <v>37</v>
       </c>
       <c r="E58" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F58" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G58">
         <v>-13.89689349</v>
@@ -2390,24 +2372,24 @@
         <v>-76.312002449999994</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B59" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C59" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D59">
         <v>38</v>
       </c>
       <c r="E59" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F59" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G59">
         <v>-14.146628400000001</v>
@@ -2416,24 +2398,24 @@
         <v>-76.26905198</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C60" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D60">
         <v>39</v>
       </c>
       <c r="E60" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F60" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G60">
         <v>-14.15086923</v>
@@ -2442,24 +2424,24 @@
         <v>-76.252262329999994</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B61" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C61" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D61">
         <v>40</v>
       </c>
       <c r="E61" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G61">
         <v>-15.3582064</v>
@@ -2468,24 +2450,24 @@
         <v>-75.161518520000001</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C62" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D62">
         <v>41</v>
       </c>
       <c r="E62" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F62" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G62">
         <v>-15.570089640000001</v>
@@ -2494,24 +2476,24 @@
         <v>-74.85327427</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B63" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C63" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D63">
         <v>42</v>
       </c>
       <c r="E63" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F63" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G63">
         <v>-15.865131030000001</v>
@@ -2520,21 +2502,21 @@
         <v>-74.249302060000005</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B64" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C64" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E64" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F64" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G64">
         <v>-15.99865842</v>
@@ -2543,24 +2525,24 @@
         <v>-74.025420980000007</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B65" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C65" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D65">
         <v>43</v>
       </c>
       <c r="E65" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F65" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G65">
         <v>-16.229926670000001</v>
@@ -2569,24 +2551,24 @@
         <v>-73.697445950000002</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B66" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C66" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D66">
         <v>44</v>
       </c>
       <c r="E66" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F66" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G66">
         <v>-16.406211129999999</v>
@@ -2595,24 +2577,24 @@
         <v>-73.220671999999993</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B67" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D67">
         <v>45</v>
       </c>
       <c r="E67" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F67" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G67">
         <v>-16.714817329999999</v>
@@ -2621,24 +2603,24 @@
         <v>-72.434944360000003</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B68" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C68" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D68">
         <v>46</v>
       </c>
       <c r="E68" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F68" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G68">
         <v>-17.015596240000001</v>
@@ -2647,24 +2629,24 @@
         <v>-72.109427960000005</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B69" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C69" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D69">
         <v>102</v>
       </c>
       <c r="E69" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F69" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G69">
         <v>-17.182473890000001</v>
@@ -2673,24 +2655,24 @@
         <v>-71.816338970000004</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B70" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C70" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D70">
         <v>47</v>
       </c>
       <c r="E70" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F70" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G70">
         <v>-17.64372921</v>
@@ -2699,24 +2681,24 @@
         <v>-71.347087000000002</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C71" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D71">
         <v>49</v>
       </c>
       <c r="E71" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F71" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G71">
         <v>-17.99395226</v>
@@ -2725,24 +2707,24 @@
         <v>-70.884207029999999</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C72" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D72">
         <v>50</v>
       </c>
       <c r="E72" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F72" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G72">
         <v>-18.117167590000001</v>
@@ -2751,24 +2733,24 @@
         <v>-70.728145249999997</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B73" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C73" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D73">
         <v>100</v>
       </c>
       <c r="E73" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F73" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G73">
         <v>-18.29689986</v>
@@ -2778,11 +2760,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H73" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H73">
-      <sortCondition descending="1" ref="G1:G73"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>